<commit_message>
Update nilai siswa otomatis
</commit_message>
<xml_diff>
--- a/nilai/data_siswa.xlsx
+++ b/nilai/data_siswa.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\web\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\web\nilai\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F32EBA32-ADA4-4B1A-B608-BE1C1742AD57}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EAD63DD7-41B7-41D6-8FDA-1853CA0BBAD8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{94B37993-57FC-457C-970B-6E7EDB0DEC76}"/>
   </bookViews>
@@ -42,9 +42,6 @@
     <t>nama</t>
   </si>
   <si>
-    <t>tgl _lahir</t>
-  </si>
-  <si>
     <t>matematika</t>
   </si>
   <si>
@@ -286,6 +283,9 @@
   </si>
   <si>
     <t>2016-10-01</t>
+  </si>
+  <si>
+    <t>tgl_lahir</t>
   </si>
 </sst>
 </file>
@@ -653,33 +653,33 @@
         <v>1</v>
       </c>
       <c r="C1" t="s">
+        <v>83</v>
+      </c>
+      <c r="D1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="E1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="F1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="G1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="H1" t="s">
         <v>6</v>
-      </c>
-      <c r="H1" t="s">
-        <v>7</v>
       </c>
     </row>
     <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
       <c r="B2" t="s">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C2" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="D2">
         <v>88</v>
@@ -699,13 +699,13 @@
     </row>
     <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
       <c r="B3" t="s">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C3" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="D3">
         <v>88</v>
@@ -725,13 +725,13 @@
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
       <c r="B4" t="s">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="C4" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="D4">
         <v>88</v>
@@ -751,13 +751,13 @@
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
       <c r="B5" t="s">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="C5" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="D5">
         <v>88</v>
@@ -777,13 +777,13 @@
     </row>
     <row r="6" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A6" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
       <c r="B6" t="s">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="C6" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="D6">
         <v>88</v>
@@ -803,13 +803,13 @@
     </row>
     <row r="7" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A7" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
       <c r="B7" t="s">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="C7" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="D7">
         <v>88</v>
@@ -829,13 +829,13 @@
     </row>
     <row r="8" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A8" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="B8" t="s">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="C8" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="D8">
         <v>88</v>
@@ -855,13 +855,13 @@
     </row>
     <row r="9" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A9" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="B9" t="s">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="C9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="D9">
         <v>88</v>
@@ -881,13 +881,13 @@
     </row>
     <row r="10" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A10" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="B10" t="s">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="C10" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="D10">
         <v>88</v>
@@ -907,13 +907,13 @@
     </row>
     <row r="11" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A11" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
       <c r="B11" t="s">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="C11" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="D11">
         <v>88</v>
@@ -933,13 +933,13 @@
     </row>
     <row r="12" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A12" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="B12" t="s">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="C12" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="D12">
         <v>88</v>
@@ -959,13 +959,13 @@
     </row>
     <row r="13" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A13" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="B13" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C13" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="D13">
         <v>88</v>
@@ -985,13 +985,13 @@
     </row>
     <row r="14" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A14" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="B14" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C14" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="D14">
         <v>88</v>
@@ -1011,13 +1011,13 @@
     </row>
     <row r="15" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A15" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="B15" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C15" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D15">
         <v>88</v>
@@ -1037,13 +1037,13 @@
     </row>
     <row r="16" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A16" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="B16" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="C16" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="D16">
         <v>88</v>
@@ -1063,13 +1063,13 @@
     </row>
     <row r="17" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A17" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="B17" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="C17" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D17">
         <v>88</v>
@@ -1089,13 +1089,13 @@
     </row>
     <row r="18" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A18" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="B18" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="C18" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="D18">
         <v>88</v>
@@ -1115,13 +1115,13 @@
     </row>
     <row r="19" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A19" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="B19" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="C19" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="D19">
         <v>88</v>
@@ -1141,13 +1141,13 @@
     </row>
     <row r="20" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A20" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="B20" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C20" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="D20">
         <v>88</v>
@@ -1167,13 +1167,13 @@
     </row>
     <row r="21" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A21" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="B21" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C21" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="D21">
         <v>88</v>
@@ -1193,13 +1193,13 @@
     </row>
     <row r="22" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A22" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="B22" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C22" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="D22">
         <v>88</v>
@@ -1219,13 +1219,13 @@
     </row>
     <row r="23" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A23" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="B23" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C23" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="D23">
         <v>88</v>
@@ -1245,13 +1245,13 @@
     </row>
     <row r="24" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A24" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="B24" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C24" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="D24">
         <v>88</v>
@@ -1271,13 +1271,13 @@
     </row>
     <row r="25" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A25" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="B25" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
       <c r="C25" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="D25">
         <v>88</v>
@@ -1297,13 +1297,13 @@
     </row>
     <row r="26" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A26" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="B26" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C26" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="D26">
         <v>88</v>
@@ -1323,13 +1323,13 @@
     </row>
     <row r="27" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A27" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="B27" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="C27" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="D27">
         <v>88</v>

</xml_diff>